<commit_message>
Apply estimator answers on overhead, supervision and burden
Office PM line kept as a dedicated per-job cost separate from the
$22/hr overhead; supervision confirmed not double counted with the
Foreman & PM crew share; labour rates confirmed fully burdened. Audit
notes updated with an Answered section.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017v7xbZSLie9k4EHji1sxso
</commit_message>
<xml_diff>
--- a/New Excel bidding Spreadsheet.xlsx
+++ b/New Excel bidding Spreadsheet.xlsx
@@ -256,7 +256,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Check for double counting: Foreman &amp; PM is already 14% of the crew mix on LABOUR RATES. Only enter supervision here if it is NOT already in the crew hours.</t>
+          <t xml:space="preserve">Confirmed: field supervision here is separate from the Foreman &amp; PM share of the crew mix, so it is not a double count.</t>
         </r>
       </text>
     </comment>
@@ -268,7 +268,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">$7,500/month from original PRJ INFO D53. The original charged this 100% to Plumbing; here it auto-splits by direct cost. Confirm it is not already inside the $22/hr overhead.</t>
+          <t xml:space="preserve">$7,500/month from original PRJ INFO D53. The original charged this 100% to Plumbing; here it auto-splits by direct cost. Confirmed: the $22/hr overhead covers salaried staff company wide; this line is the PM assigned to this job, so it is not a double count.</t>
         </r>
       </text>
     </comment>
@@ -299,7 +299,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1523" uniqueCount="737">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1527" uniqueCount="739">
   <si>
     <t xml:space="preserve">New Excel Bidding Spreadsheet: How It Works</t>
   </si>
@@ -820,7 +820,7 @@
     <t xml:space="preserve">Apprentice Lvl 1-2</t>
   </si>
   <si>
-    <t xml:space="preserve">Rates are average hourly W/ burden (from original PRJ INFO D36:D40).</t>
+    <t xml:space="preserve">Rates are fully burdened (confirmed): from original PRJ INFO D36:D40.</t>
   </si>
   <si>
     <t xml:space="preserve">Apprentice Lvl 3-6</t>
@@ -1504,10 +1504,10 @@
     <t xml:space="preserve">Supervision - A/C</t>
   </si>
   <si>
-    <t xml:space="preserve">Office Management (PM / estimating / admin)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">From PRJ INFO D53 'Office MGMT CTGCY'</t>
+    <t xml:space="preserve">Office Project Manager (dedicated to this job)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dedicated office PM, per month</t>
   </si>
   <si>
     <t xml:space="preserve">Bonus - Plumbing</t>
@@ -2368,10 +2368,10 @@
     <t xml:space="preserve">$7,500/month x 24 months = $180,000 (+15% = $207,000) is allocated 100% to Plumbing, using the HVAC duration.</t>
   </si>
   <si>
-    <t xml:space="preserve">Plumbing looks $207,000 more expensive than it is; HVAC looks cheaper. Also check it is not already inside the $22/hr overhead.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Office Management auto-splits by direct cost (or set your own %). Flagged for double-count review.</t>
+    <t xml:space="preserve">Plumbing looks $207,000 more expensive than it is; HVAC looks cheaper. Confirmed this is a real job cost (dedicated PM), separate from the $22/hr overhead.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kept as 'Office Project Manager'. Auto-splits by direct cost across divisions (or set your own %).</t>
   </si>
   <si>
     <t xml:space="preserve">PRJ SUMMARY M55:T79 ("50-50 Div's" split)</t>
@@ -2449,16 +2449,19 @@
     <t xml:space="preserve">Kept on both tabs, labelled 'if by Plumbing' / 'if by HVAC'. Use only one.</t>
   </si>
   <si>
+    <t xml:space="preserve">OK</t>
+  </si>
+  <si>
     <t xml:space="preserve">PRJ INFO E40 (Foreman &amp; PM 14%) and PRJ SUMMARY rows 55-58</t>
   </si>
   <si>
     <t xml:space="preserve">Foreman &amp; PM time is in the crew mix and supervision is also a GC line.</t>
   </si>
   <si>
-    <t xml:space="preserve">Possible double count of supervision.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comment on SUBS &amp; GC supervision rows; question for you below.</t>
+    <t xml:space="preserve">Reviewed with estimator: these are separate costs, not a double count.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both kept: crew mix on LABOUR RATES, supervision on SUBS &amp; GC.</t>
   </si>
   <si>
     <t xml:space="preserve">BUDGET PLAN J1</t>
@@ -2488,15 +2491,6 @@
     <t xml:space="preserve">OPEN QUESTIONS FOR YOU</t>
   </si>
   <si>
-    <t xml:space="preserve">Is the $22/hr overhead meant to cover office management ($7,500/month)? If yes, delete the Office Management GC line to avoid double counting.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Is Foreman &amp; PM time already in the 14% crew mix? If yes, leave the Supervision GC rows at $0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Are the 'Average hourly rates W/ burden' fully burdened (CPP, EI, WCB, vacation, benefits, union dues)? If not, what burden % should be added?</t>
-  </si>
-  <si>
     <t xml:space="preserve">Target margin per division (placeholder is 15%). Do subs carry a lower margin than self-perform work?</t>
   </si>
   <si>
@@ -2510,6 +2504,18 @@
   </si>
   <si>
     <t xml:space="preserve">Do the price-list and takeoff tabs (P&amp;H MATERIAL, HVAC MATERIAL, EQUIPMENT) need to come across, or will takeoff totals be typed in as Qty x unit cost?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANSWERED (decisions built into this workbook)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$22/hr overhead covers all salaried staff company wide. A dedicated office project manager per job is a separate monthly cost, so the Office Project Manager GC line stays.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Field supervision GC lines are not double counted with the Foreman &amp; PM share of the crew mix. Both stay.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labour rates on LABOUR RATES are fully burdened (CPP, EI, WCB, vacation, benefits). No extra burden % is added.</t>
   </si>
 </sst>
 </file>
@@ -2529,7 +2535,7 @@
     <numFmt numFmtId="173" formatCode="0%;;&quot;&quot;"/>
     <numFmt numFmtId="174" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2665,6 +2671,14 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF006100"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -2766,7 +2780,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="90">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3111,12 +3125,20 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -8054,7 +8076,7 @@
     <tabColor rgb="FF7F7F7F"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -8398,20 +8420,20 @@
       <c r="A20" s="81" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="85" t="s">
-        <v>707</v>
+      <c r="B20" s="86" t="s">
+        <v>716</v>
       </c>
       <c r="C20" s="83" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="D20" s="83" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="E20" s="83" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="F20" s="83" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8422,16 +8444,16 @@
         <v>707</v>
       </c>
       <c r="C21" s="83" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="D21" s="83" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="E21" s="83" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="F21" s="83" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8442,110 +8464,115 @@
         <v>707</v>
       </c>
       <c r="C22" s="83" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="D22" s="83" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="E22" s="83" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="F22" s="83" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="3" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="86" t="n">
+      <c r="B26" s="87" t="n">
         <v>1</v>
       </c>
-      <c r="C26" s="87" t="s">
-        <v>729</v>
-      </c>
-      <c r="D26" s="87"/>
-      <c r="E26" s="87"/>
-      <c r="F26" s="87"/>
+      <c r="C26" s="88" t="s">
+        <v>730</v>
+      </c>
+      <c r="D26" s="88"/>
+      <c r="E26" s="88"/>
+      <c r="F26" s="88"/>
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="86" t="n">
+      <c r="B27" s="87" t="n">
         <v>2</v>
       </c>
-      <c r="C27" s="87" t="s">
-        <v>730</v>
-      </c>
-      <c r="D27" s="87"/>
-      <c r="E27" s="87"/>
-      <c r="F27" s="87"/>
+      <c r="C27" s="88" t="s">
+        <v>731</v>
+      </c>
+      <c r="D27" s="88"/>
+      <c r="E27" s="88"/>
+      <c r="F27" s="88"/>
     </row>
     <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="86" t="n">
+      <c r="B28" s="87" t="n">
         <v>3</v>
       </c>
-      <c r="C28" s="87" t="s">
-        <v>731</v>
-      </c>
-      <c r="D28" s="87"/>
-      <c r="E28" s="87"/>
-      <c r="F28" s="87"/>
+      <c r="C28" s="88" t="s">
+        <v>732</v>
+      </c>
+      <c r="D28" s="88"/>
+      <c r="E28" s="88"/>
+      <c r="F28" s="88"/>
     </row>
     <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="86" t="n">
+      <c r="B29" s="87" t="n">
         <v>4</v>
       </c>
-      <c r="C29" s="87" t="s">
-        <v>732</v>
-      </c>
-      <c r="D29" s="87"/>
-      <c r="E29" s="87"/>
-      <c r="F29" s="87"/>
+      <c r="C29" s="88" t="s">
+        <v>733</v>
+      </c>
+      <c r="D29" s="88"/>
+      <c r="E29" s="88"/>
+      <c r="F29" s="88"/>
     </row>
     <row r="30" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="86" t="n">
+      <c r="B30" s="87" t="n">
         <v>5</v>
       </c>
-      <c r="C30" s="87" t="s">
-        <v>733</v>
-      </c>
-      <c r="D30" s="87"/>
-      <c r="E30" s="87"/>
-      <c r="F30" s="87"/>
-    </row>
-    <row r="31" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="86" t="n">
-        <v>6</v>
-      </c>
-      <c r="C31" s="87" t="s">
+      <c r="C30" s="88" t="s">
         <v>734</v>
       </c>
-      <c r="D31" s="87"/>
-      <c r="E31" s="87"/>
-      <c r="F31" s="87"/>
-    </row>
-    <row r="32" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="86" t="n">
-        <v>7</v>
-      </c>
-      <c r="C32" s="87" t="s">
+      <c r="D30" s="88"/>
+      <c r="E30" s="88"/>
+      <c r="F30" s="88"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="3" t="s">
         <v>735</v>
       </c>
-      <c r="D32" s="87"/>
-      <c r="E32" s="87"/>
-      <c r="F32" s="87"/>
     </row>
     <row r="33" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="86" t="n">
-        <v>8</v>
-      </c>
-      <c r="C33" s="87" t="s">
+      <c r="B33" s="89" t="s">
+        <v>716</v>
+      </c>
+      <c r="C33" s="88" t="s">
         <v>736</v>
       </c>
-      <c r="D33" s="87"/>
-      <c r="E33" s="87"/>
-      <c r="F33" s="87"/>
+      <c r="D33" s="88"/>
+      <c r="E33" s="88"/>
+      <c r="F33" s="88"/>
+    </row>
+    <row r="34" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="89" t="s">
+        <v>716</v>
+      </c>
+      <c r="C34" s="88" t="s">
+        <v>737</v>
+      </c>
+      <c r="D34" s="88"/>
+      <c r="E34" s="88"/>
+      <c r="F34" s="88"/>
+    </row>
+    <row r="35" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="89" t="s">
+        <v>716</v>
+      </c>
+      <c r="C35" s="88" t="s">
+        <v>738</v>
+      </c>
+      <c r="D35" s="88"/>
+      <c r="E35" s="88"/>
+      <c r="F35" s="88"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -8554,9 +8581,9 @@
     <mergeCell ref="C28:F28"/>
     <mergeCell ref="C29:F29"/>
     <mergeCell ref="C30:F30"/>
-    <mergeCell ref="C31:F31"/>
-    <mergeCell ref="C32:F32"/>
     <mergeCell ref="C33:F33"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C35:F35"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>